<commit_message>
Add proxy on backend to make Mercado Pago work
</commit_message>
<xml_diff>
--- a/backend/master_workbook.xlsx
+++ b/backend/master_workbook.xlsx
@@ -520,7 +520,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F78"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
@@ -2340,7 +2340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4295,6 +4295,47 @@
         <v>0</v>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>20260810033028223048</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-08-10T03:30:28.223048+00:00</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>SALE</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>S004</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>PIX</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H47" t="n">
+        <v>1</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>